<commit_message>
Sync planning SharePoint : S16
</commit_message>
<xml_diff>
--- a/Plannings 2026 S16.xlsx
+++ b/Plannings 2026 S16.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{85468703-40F4-4AB4-B59D-9AA85ACBEEF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{85468703-40F4-4AB4-B59D-9AA85ACBEEF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3A5B07A-8FED-4E31-BA69-31D742EA78EE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="145">
   <si>
     <t>Planning des salariés du 13/04/2026 au 19/04/2026</t>
   </si>
@@ -451,6 +451,12 @@
   </si>
   <si>
     <t>LOUIBA Yacine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. PADEL // </t>
+  </si>
+  <si>
+    <t>P50M // ANIV</t>
   </si>
 </sst>
 </file>
@@ -846,7 +852,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -956,9 +962,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -981,9 +984,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1026,6 +1026,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5675,13 +5684,17 @@
       <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="15"/>
+      <c r="B3" s="15" t="s">
+        <v>143</v>
+      </c>
       <c r="C3" s="15"/>
       <c r="D3" s="15"/>
       <c r="E3" s="15"/>
       <c r="F3" s="15"/>
       <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
+      <c r="H3" s="15" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
@@ -5801,16 +5814,16 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="24"/>
-      <c r="B11" s="47" t="s">
+      <c r="B11" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="47" t="s">
+      <c r="C11" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="47" t="s">
+      <c r="D11" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="44" t="s">
+      <c r="E11" s="43" t="s">
         <v>23</v>
       </c>
       <c r="F11" s="1"/>
@@ -5819,16 +5832,16 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="24"/>
-      <c r="B12" s="48" t="s">
+      <c r="B12" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="48" t="s">
+      <c r="C12" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="48" t="s">
+      <c r="D12" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="42" t="s">
+      <c r="E12" s="41" t="s">
         <v>27</v>
       </c>
       <c r="F12" s="1"/>
@@ -5840,13 +5853,13 @@
       <c r="B13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="47" t="s">
+      <c r="C13" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="44" t="s">
+      <c r="D13" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="42"/>
+      <c r="E13" s="41"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="25"/>
@@ -5856,13 +5869,13 @@
       <c r="B14" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="50" t="s">
+      <c r="C14" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="43"/>
+      <c r="E14" s="42"/>
       <c r="F14" s="22"/>
       <c r="G14" s="22"/>
       <c r="H14" s="23"/>
@@ -5879,7 +5892,7 @@
       <c r="E15" s="18"/>
       <c r="F15" s="18"/>
       <c r="G15" s="18"/>
-      <c r="H15" s="36" t="s">
+      <c r="H15" s="44" t="s">
         <v>29</v>
       </c>
     </row>
@@ -5893,7 +5906,7 @@
       <c r="E16" s="22"/>
       <c r="F16" s="22"/>
       <c r="G16" s="22"/>
-      <c r="H16" s="37" t="s">
+      <c r="H16" s="61" t="s">
         <v>35</v>
       </c>
     </row>
@@ -5964,7 +5977,7 @@
       <c r="F20" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="G20" s="60" t="s">
+      <c r="G20" s="58" t="s">
         <v>43</v>
       </c>
       <c r="H20" s="19"/>
@@ -5980,7 +5993,7 @@
       <c r="F21" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G21" s="59" t="s">
+      <c r="G21" s="57" t="s">
         <v>46</v>
       </c>
       <c r="H21" s="25"/>
@@ -6013,41 +6026,41 @@
       <c r="A24" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="52" t="s">
+      <c r="B24" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="52" t="s">
+      <c r="C24" s="50" t="s">
         <v>49</v>
       </c>
       <c r="D24" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="E24" s="41" t="s">
+      <c r="E24" s="40" t="s">
         <v>23</v>
       </c>
       <c r="F24" s="18"/>
       <c r="G24" s="18"/>
-      <c r="H24" s="45" t="s">
+      <c r="H24" s="59" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="24"/>
-      <c r="B25" s="53" t="s">
+      <c r="B25" s="51" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="53" t="s">
+      <c r="C25" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="38" t="s">
+      <c r="D25" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E25" s="42" t="s">
+      <c r="E25" s="41" t="s">
         <v>27</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
-      <c r="H25" s="46" t="s">
+      <c r="H25" s="60" t="s">
         <v>53</v>
       </c>
     </row>
@@ -6059,10 +6072,10 @@
       <c r="C26" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="39" t="s">
+      <c r="D26" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="E26" s="42"/>
+      <c r="E26" s="41"/>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="31" t="s">
@@ -6077,10 +6090,10 @@
       <c r="C27" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="38" t="s">
+      <c r="D27" s="37" t="s">
         <v>58</v>
       </c>
-      <c r="E27" s="42"/>
+      <c r="E27" s="41"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="25" t="s">
@@ -6089,76 +6102,76 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="24"/>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="51" t="s">
+      <c r="C28" s="49" t="s">
         <v>49</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E28" s="42"/>
+      <c r="E28" s="41"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="25"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="24"/>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="53" t="s">
+      <c r="C29" s="51" t="s">
         <v>61</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E29" s="42"/>
+      <c r="E29" s="41"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="25"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="24"/>
-      <c r="B30" s="39" t="s">
+      <c r="B30" s="38" t="s">
         <v>49</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D30" s="51" t="s">
+      <c r="D30" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="E30" s="42"/>
+      <c r="E30" s="41"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="25"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="24"/>
-      <c r="B31" s="38" t="s">
+      <c r="B31" s="37" t="s">
         <v>63</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="53" t="s">
+      <c r="D31" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="E31" s="42"/>
+      <c r="E31" s="41"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="25"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="24"/>
-      <c r="B32" s="38"/>
-      <c r="C32" s="51" t="s">
+      <c r="B32" s="37"/>
+      <c r="C32" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="D32" s="38"/>
-      <c r="E32" s="42"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="41"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="25"/>
@@ -6170,7 +6183,7 @@
         <v>66</v>
       </c>
       <c r="D33" s="35"/>
-      <c r="E33" s="43"/>
+      <c r="E33" s="42"/>
       <c r="F33" s="22"/>
       <c r="G33" s="22"/>
       <c r="H33" s="23"/>
@@ -6225,7 +6238,7 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="24"/>
-      <c r="B37" s="38" t="s">
+      <c r="B37" s="37" t="s">
         <v>20</v>
       </c>
       <c r="C37" s="1"/>
@@ -6235,21 +6248,21 @@
       <c r="E37" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F37" s="38" t="s">
+      <c r="F37" s="37" t="s">
         <v>20</v>
       </c>
       <c r="G37" s="1"/>
-      <c r="H37" s="40" t="s">
+      <c r="H37" s="39" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="24"/>
-      <c r="B38" s="44" t="s">
+      <c r="B38" s="43" t="s">
         <v>73</v>
       </c>
       <c r="C38" s="1"/>
-      <c r="D38" s="39" t="s">
+      <c r="D38" s="38" t="s">
         <v>74</v>
       </c>
       <c r="E38" s="1"/>
@@ -6257,17 +6270,17 @@
         <v>15</v>
       </c>
       <c r="G38" s="1"/>
-      <c r="H38" s="56" t="s">
+      <c r="H38" s="54" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
-      <c r="B39" s="42" t="s">
+      <c r="B39" s="41" t="s">
         <v>76</v>
       </c>
       <c r="C39" s="1"/>
-      <c r="D39" s="38" t="s">
+      <c r="D39" s="37" t="s">
         <v>58</v>
       </c>
       <c r="E39" s="1"/>
@@ -6275,13 +6288,13 @@
         <v>77</v>
       </c>
       <c r="G39" s="1"/>
-      <c r="H39" s="57" t="s">
+      <c r="H39" s="55" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="24"/>
-      <c r="B40" s="42"/>
+      <c r="B40" s="41"/>
       <c r="C40" s="1"/>
       <c r="D40" s="2" t="s">
         <v>15</v>
@@ -6295,7 +6308,7 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="24"/>
-      <c r="B41" s="42"/>
+      <c r="B41" s="41"/>
       <c r="C41" s="1"/>
       <c r="D41" s="1" t="s">
         <v>79</v>
@@ -6309,9 +6322,9 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="24"/>
-      <c r="B42" s="42"/>
+      <c r="B42" s="41"/>
       <c r="C42" s="1"/>
-      <c r="D42" s="39" t="s">
+      <c r="D42" s="38" t="s">
         <v>74</v>
       </c>
       <c r="E42" s="1"/>
@@ -6321,7 +6334,7 @@
     </row>
     <row r="43" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="20"/>
-      <c r="B43" s="43"/>
+      <c r="B43" s="42"/>
       <c r="C43" s="22"/>
       <c r="D43" s="35" t="s">
         <v>81</v>
@@ -6399,13 +6412,13 @@
       <c r="A49" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="B49" s="49" t="s">
+      <c r="B49" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="C49" s="49" t="s">
+      <c r="C49" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="D49" s="49" t="s">
+      <c r="D49" s="47" t="s">
         <v>28</v>
       </c>
       <c r="E49" s="18"/>
@@ -6415,13 +6428,13 @@
     </row>
     <row r="50" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="30"/>
-      <c r="B50" s="48" t="s">
+      <c r="B50" s="46" t="s">
         <v>85</v>
       </c>
-      <c r="C50" s="48" t="s">
+      <c r="C50" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="D50" s="48" t="s">
+      <c r="D50" s="46" t="s">
         <v>85</v>
       </c>
       <c r="E50" s="1"/>
@@ -6439,7 +6452,7 @@
       <c r="E51" s="18"/>
       <c r="F51" s="18"/>
       <c r="G51" s="18"/>
-      <c r="H51" s="54" t="s">
+      <c r="H51" s="52" t="s">
         <v>43</v>
       </c>
     </row>
@@ -6451,7 +6464,7 @@
       <c r="E52" s="22"/>
       <c r="F52" s="22"/>
       <c r="G52" s="22"/>
-      <c r="H52" s="55" t="s">
+      <c r="H52" s="53" t="s">
         <v>91</v>
       </c>
     </row>
@@ -6515,7 +6528,7 @@
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
-      <c r="H57" s="56" t="s">
+      <c r="H57" s="54" t="s">
         <v>43</v>
       </c>
     </row>
@@ -6527,7 +6540,7 @@
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
       <c r="G58" s="1"/>
-      <c r="H58" s="57" t="s">
+      <c r="H58" s="55" t="s">
         <v>95</v>
       </c>
     </row>
@@ -6563,7 +6576,7 @@
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
-      <c r="H61" s="56" t="s">
+      <c r="H61" s="54" t="s">
         <v>43</v>
       </c>
     </row>
@@ -6575,7 +6588,7 @@
       <c r="E62" s="22"/>
       <c r="F62" s="22"/>
       <c r="G62" s="22"/>
-      <c r="H62" s="55" t="s">
+      <c r="H62" s="53" t="s">
         <v>97</v>
       </c>
     </row>
@@ -6611,7 +6624,7 @@
       <c r="G64" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="H64" s="19" t="s">
+      <c r="H64" s="36" t="s">
         <v>69</v>
       </c>
     </row>
@@ -6620,27 +6633,27 @@
       <c r="B65" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C65" s="38" t="s">
+      <c r="C65" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="D65" s="38" t="s">
+      <c r="D65" s="37" t="s">
         <v>91</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>101</v>
       </c>
       <c r="F65" s="1"/>
-      <c r="G65" s="38" t="s">
+      <c r="G65" s="37" t="s">
         <v>102</v>
       </c>
-      <c r="H65" s="25" t="s">
+      <c r="H65" s="39" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="24"/>
       <c r="B66" s="1"/>
-      <c r="C66" s="47" t="s">
+      <c r="C66" s="45" t="s">
         <v>28</v>
       </c>
       <c r="D66" s="2" t="s">
@@ -6648,15 +6661,15 @@
       </c>
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
-      <c r="G66" s="39" t="s">
+      <c r="G66" s="38" t="s">
         <v>74</v>
       </c>
-      <c r="H66" s="25"/>
+      <c r="H66" s="39"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="24"/>
       <c r="B67" s="1"/>
-      <c r="C67" s="48" t="s">
+      <c r="C67" s="46" t="s">
         <v>85</v>
       </c>
       <c r="D67" s="1" t="s">
@@ -6664,62 +6677,62 @@
       </c>
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
-      <c r="G67" s="38" t="s">
+      <c r="G67" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="H67" s="25"/>
+      <c r="H67" s="39"/>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="24"/>
       <c r="B68" s="1"/>
-      <c r="C68" s="48"/>
-      <c r="D68" s="47" t="s">
+      <c r="C68" s="46"/>
+      <c r="D68" s="45" t="s">
         <v>28</v>
       </c>
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
-      <c r="G68" s="39" t="s">
+      <c r="G68" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="H68" s="25"/>
+      <c r="H68" s="39"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="24"/>
       <c r="B69" s="1"/>
-      <c r="C69" s="48"/>
-      <c r="D69" s="48" t="s">
+      <c r="C69" s="46"/>
+      <c r="D69" s="46" t="s">
         <v>31</v>
       </c>
       <c r="E69" s="1"/>
       <c r="F69" s="1"/>
-      <c r="G69" s="38" t="s">
+      <c r="G69" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="H69" s="25"/>
+      <c r="H69" s="39"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="24"/>
       <c r="B70" s="1"/>
-      <c r="C70" s="48"/>
-      <c r="D70" s="48"/>
+      <c r="C70" s="46"/>
+      <c r="D70" s="46"/>
       <c r="E70" s="1"/>
       <c r="F70" s="1"/>
-      <c r="G70" s="58" t="s">
+      <c r="G70" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="H70" s="25"/>
+      <c r="H70" s="39"/>
     </row>
     <row r="71" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="30"/>
       <c r="B71" s="1"/>
-      <c r="C71" s="48"/>
-      <c r="D71" s="48"/>
+      <c r="C71" s="46"/>
+      <c r="D71" s="46"/>
       <c r="E71" s="1"/>
       <c r="F71" s="1"/>
-      <c r="G71" s="59" t="s">
+      <c r="G71" s="57" t="s">
         <v>107</v>
       </c>
-      <c r="H71" s="25"/>
+      <c r="H71" s="39"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="16" t="s">
@@ -6795,7 +6808,7 @@
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="24"/>
-      <c r="B76" s="44" t="s">
+      <c r="B76" s="43" t="s">
         <v>73</v>
       </c>
       <c r="C76" s="1"/>
@@ -6809,7 +6822,7 @@
     </row>
     <row r="77" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="20"/>
-      <c r="B77" s="43" t="s">
+      <c r="B77" s="42" t="s">
         <v>115</v>
       </c>
       <c r="C77" s="22"/>
@@ -6825,7 +6838,7 @@
       <c r="A78" s="33" t="s">
         <v>117</v>
       </c>
-      <c r="B78" s="48" t="s">
+      <c r="B78" s="46" t="s">
         <v>28</v>
       </c>
       <c r="C78" s="1"/>
@@ -6839,7 +6852,7 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="24"/>
-      <c r="B79" s="48" t="s">
+      <c r="B79" s="46" t="s">
         <v>85</v>
       </c>
       <c r="C79" s="1"/>
@@ -6853,31 +6866,31 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="24"/>
-      <c r="B80" s="48"/>
+      <c r="B80" s="46"/>
       <c r="C80" s="1"/>
       <c r="D80" s="1"/>
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
-      <c r="G80" s="58" t="s">
+      <c r="G80" s="56" t="s">
         <v>43</v>
       </c>
       <c r="H80" s="25"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="24"/>
-      <c r="B81" s="48"/>
+      <c r="B81" s="46"/>
       <c r="C81" s="1"/>
       <c r="D81" s="1"/>
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
-      <c r="G81" s="59" t="s">
+      <c r="G81" s="57" t="s">
         <v>91</v>
       </c>
       <c r="H81" s="25"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="24"/>
-      <c r="B82" s="48"/>
+      <c r="B82" s="46"/>
       <c r="C82" s="1"/>
       <c r="D82" s="1"/>
       <c r="E82" s="1"/>
@@ -6889,7 +6902,7 @@
     </row>
     <row r="83" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="20"/>
-      <c r="B83" s="50"/>
+      <c r="B83" s="48"/>
       <c r="C83" s="22"/>
       <c r="D83" s="22"/>
       <c r="E83" s="22"/>
@@ -6946,7 +6959,7 @@
       <c r="D87" s="1"/>
       <c r="E87" s="1"/>
       <c r="F87" s="1"/>
-      <c r="G87" s="38" t="s">
+      <c r="G87" s="37" t="s">
         <v>13</v>
       </c>
       <c r="H87" s="25"/>
@@ -6958,7 +6971,7 @@
       <c r="D88" s="1"/>
       <c r="E88" s="1"/>
       <c r="F88" s="1"/>
-      <c r="G88" s="39" t="s">
+      <c r="G88" s="38" t="s">
         <v>12</v>
       </c>
       <c r="H88" s="25"/>
@@ -6999,7 +7012,7 @@
         <v>15</v>
       </c>
       <c r="E91" s="18"/>
-      <c r="F91" s="41" t="s">
+      <c r="F91" s="40" t="s">
         <v>29</v>
       </c>
       <c r="G91" s="18"/>
@@ -7015,7 +7028,7 @@
         <v>16</v>
       </c>
       <c r="E92" s="22"/>
-      <c r="F92" s="43" t="s">
+      <c r="F92" s="42" t="s">
         <v>126</v>
       </c>
       <c r="G92" s="22"/>
@@ -7839,13 +7852,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6EC8FFF-5362-4FBB-81C5-0CE8BAD24C7B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8F6C438-A15A-4C89-91F4-58B83B61C682}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38A3F63F-2F60-43C0-8654-FD02CB6B1CD3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D3BE358-601C-4399-86C5-69B11AA2ED05}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D517EF44-A622-466A-86B4-50F7F9D79E76}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5F73B29-8E6B-4B7B-8C47-AC6D8321E5BA}"/>
 </file>
</xml_diff>